<commit_message>
Joint tracker: add Watchlist sheet (Quality @ 200-day buy zone + re-buy watch)
24 names with 200-day buy zone, buy target, review level, analyst upside,
reward:risk and a formula status. Zone and entry offsets are inputs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XBawetM5mpZm52AQxpa6eR
</commit_message>
<xml_diff>
--- a/joint_portfolio_tracker.xlsx
+++ b/joint_portfolio_tracker.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holdings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Holdings'!$A$5:$AP$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Watchlist'!$A$4:$AD$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -111,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,10 +141,11 @@
     <xf numFmtId="169" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4176,7 +4179,3063 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:AD30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="9" customWidth="1" min="27" max="27"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="34" customWidth="1" min="29" max="29"/>
+    <col width="60" customWidth="1" min="30" max="30"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Joint Watchlist - Quality @ 200-day Buy Zone + Re-buy Watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ordered by pre-breakout chart setup (most pulled back first). Blue = inputs (10/29 close), green headers = formulas. A status is a prompt to research, never a buy order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>List</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Held?</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Quality Grade</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Quality Rank</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Chart Setup</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Valuation</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Disruption</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>50-day SMA</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>200-day SMA</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Analyst Mean Target</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t># Buy</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t># Hold</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t># Sell</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>Next Earnings</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Wash-Sale Clear</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>vs 200-day</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>vs 50-day</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>Buy Zone Low</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>Buy Zone High</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>BUY TARGET</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>Distance to Buy Target</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>Upside: Buy Tgt to Analyst</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>WATCH REVIEW LEVEL</t>
+        </is>
+      </c>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>Reward : Risk at Buy Tgt</t>
+        </is>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>% Buy Ratings</t>
+        </is>
+      </c>
+      <c r="AC4" s="4" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>AEM</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Agnico Eagle Mines</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>57 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>RICH -23% (low)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>175.92</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>193.8</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>189.53</v>
+      </c>
+      <c r="M5" s="7" t="n">
+        <v>225.4</v>
+      </c>
+      <c r="N5" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="O5" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>Feb 11 (unverified)</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="n"/>
+      <c r="S5" s="12">
+        <f>J5/L5-1</f>
+        <v/>
+      </c>
+      <c r="T5" s="12">
+        <f>J5/K5-1</f>
+        <v/>
+      </c>
+      <c r="U5" s="9">
+        <f>L5*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V5" s="9">
+        <f>L5*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W5" s="9">
+        <f>L5*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X5" s="12">
+        <f>J5/W5-1</f>
+        <v/>
+      </c>
+      <c r="Y5" s="12">
+        <f>IF(N(M5)&gt;0,M5/W5-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z5" s="9">
+        <f>U5</f>
+        <v/>
+      </c>
+      <c r="AA5" s="15">
+        <f>IFERROR(IF(N(M5)&gt;W5,(M5-W5)/(W5-Z5),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB5" s="24">
+        <f>IFERROR(N5/(N5+O5+P5),"")</f>
+        <v/>
+      </c>
+      <c r="AC5" s="16">
+        <f>IF(D5="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R5),Inputs!$B$5&lt;R5,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R5,"m/d"),IF(J5&lt;U5,"BELOW ZONE: wait for 200-day reclaim",IF(J5&gt;V5,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q5),AND(Q5&gt;Inputs!$B$5,Q5-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M5)&lt;=J5,"IN ZONE: analysts see no upside",IF(J5&lt;=W5,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD5" s="17" t="inlineStr">
+        <is>
+          <t>Falling wedge forming; tracks gold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Seagate</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>57 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -50% (low)</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>700.47</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>803.15</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>690.92</v>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>1062.55</v>
+      </c>
+      <c r="N6" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="O6" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>Jan 26 (unverified)</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="n"/>
+      <c r="S6" s="12">
+        <f>J6/L6-1</f>
+        <v/>
+      </c>
+      <c r="T6" s="12">
+        <f>J6/K6-1</f>
+        <v/>
+      </c>
+      <c r="U6" s="9">
+        <f>L6*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V6" s="9">
+        <f>L6*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W6" s="9">
+        <f>L6*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X6" s="12">
+        <f>J6/W6-1</f>
+        <v/>
+      </c>
+      <c r="Y6" s="12">
+        <f>IF(N(M6)&gt;0,M6/W6-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z6" s="9">
+        <f>U6</f>
+        <v/>
+      </c>
+      <c r="AA6" s="15">
+        <f>IFERROR(IF(N(M6)&gt;W6,(M6-W6)/(W6-Z6),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB6" s="24">
+        <f>IFERROR(N6/(N6+O6+P6),"")</f>
+        <v/>
+      </c>
+      <c r="AC6" s="16">
+        <f>IF(D6="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R6),Inputs!$B$5&lt;R6,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R6,"m/d"),IF(J6&lt;U6,"BELOW ZONE: wait for 200-day reclaim",IF(J6&gt;V6,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q6),AND(Q6&gt;Inputs!$B$5,Q6-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M6)&lt;=J6,"IN ZONE: analysts see no upside",IF(J6&lt;=W6,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD6" s="17" t="inlineStr">
+        <is>
+          <t>Falling wedge forming; -4.1% after hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Broadcom</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>57 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -50% (med)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>345</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>353.7</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>367.78</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>532.3099999999999</v>
+      </c>
+      <c r="N7" s="23" t="n">
+        <v>53</v>
+      </c>
+      <c r="O7" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="8" t="n">
+        <v>46365</v>
+      </c>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="12">
+        <f>J7/L7-1</f>
+        <v/>
+      </c>
+      <c r="T7" s="12">
+        <f>J7/K7-1</f>
+        <v/>
+      </c>
+      <c r="U7" s="9">
+        <f>L7*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V7" s="9">
+        <f>L7*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W7" s="9">
+        <f>L7*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X7" s="12">
+        <f>J7/W7-1</f>
+        <v/>
+      </c>
+      <c r="Y7" s="12">
+        <f>IF(N(M7)&gt;0,M7/W7-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z7" s="9">
+        <f>U7</f>
+        <v/>
+      </c>
+      <c r="AA7" s="15">
+        <f>IFERROR(IF(N(M7)&gt;W7,(M7-W7)/(W7-Z7),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB7" s="24">
+        <f>IFERROR(N7/(N7+O7+P7),"")</f>
+        <v/>
+      </c>
+      <c r="AC7" s="16">
+        <f>IF(D7="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R7),Inputs!$B$5&lt;R7,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R7,"m/d"),IF(J7&lt;U7,"BELOW ZONE: wait for 200-day reclaim",IF(J7&gt;V7,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q7),AND(Q7&gt;Inputs!$B$5,Q7-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M7)&lt;=J7,"IN ZONE: analysts see no upside",IF(J7&lt;=W7,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD7" s="17" t="inlineStr">
+        <is>
+          <t>Falling wedge forming; thesis intact 9/30. -3.7% after hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>FAIR +5% (med)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>213.66</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>221.99</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>204.28</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>334.45</v>
+      </c>
+      <c r="N8" s="23" t="n">
+        <v>69</v>
+      </c>
+      <c r="O8" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="8" t="n">
+        <v>46343</v>
+      </c>
+      <c r="R8" s="5" t="n"/>
+      <c r="S8" s="12">
+        <f>J8/L8-1</f>
+        <v/>
+      </c>
+      <c r="T8" s="12">
+        <f>J8/K8-1</f>
+        <v/>
+      </c>
+      <c r="U8" s="9">
+        <f>L8*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V8" s="9">
+        <f>L8*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W8" s="9">
+        <f>L8*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X8" s="12">
+        <f>J8/W8-1</f>
+        <v/>
+      </c>
+      <c r="Y8" s="12">
+        <f>IF(N(M8)&gt;0,M8/W8-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z8" s="9">
+        <f>U8</f>
+        <v/>
+      </c>
+      <c r="AA8" s="15">
+        <f>IFERROR(IF(N(M8)&gt;W8,(M8-W8)/(W8-Z8),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB8" s="24">
+        <f>IFERROR(N8/(N8+O8+P8),"")</f>
+        <v/>
+      </c>
+      <c r="AC8" s="16">
+        <f>IF(D8="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R8),Inputs!$B$5&lt;R8,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R8,"m/d"),IF(J8&lt;U8,"BELOW ZONE: wait for 200-day reclaim",IF(J8&gt;V8,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q8),AND(Q8&gt;Inputs!$B$5,Q8-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M8)&lt;=J8,"IN ZONE: analysts see no upside",IF(J8&lt;=W8,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD8" s="17" t="inlineStr">
+        <is>
+          <t>#1 on business quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>WES</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Western Midstream</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>RICH -19% (high)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>45.82</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>44.12</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>49.54</v>
+      </c>
+      <c r="N9" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O9" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="P9" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="8" t="n">
+        <v>46330</v>
+      </c>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="12">
+        <f>J9/L9-1</f>
+        <v/>
+      </c>
+      <c r="T9" s="12">
+        <f>J9/K9-1</f>
+        <v/>
+      </c>
+      <c r="U9" s="9">
+        <f>L9*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V9" s="9">
+        <f>L9*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W9" s="9">
+        <f>L9*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X9" s="12">
+        <f>J9/W9-1</f>
+        <v/>
+      </c>
+      <c r="Y9" s="12">
+        <f>IF(N(M9)&gt;0,M9/W9-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z9" s="9">
+        <f>U9</f>
+        <v/>
+      </c>
+      <c r="AA9" s="15">
+        <f>IFERROR(IF(N(M9)&gt;W9,(M9-W9)/(W9-Z9),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB9" s="24">
+        <f>IFERROR(N9/(N9+O9+P9),"")</f>
+        <v/>
+      </c>
+      <c r="AC9" s="16">
+        <f>IF(D9="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R9),Inputs!$B$5&lt;R9,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R9,"m/d"),IF(J9&lt;U9,"BELOW ZONE: wait for 200-day reclaim",IF(J9&gt;V9,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q9),AND(Q9&gt;Inputs!$B$5,Q9-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M9)&lt;=J9,"IN ZONE: analysts see no upside",IF(J9&lt;=W9,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD9" s="17" t="inlineStr">
+        <is>
+          <t>Double bottom near trigger 46.42. Analysts mostly Hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>SCCO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Southern Copper</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -40% (high)</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>INNOVATING</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>191.75</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>201.33</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>189.09</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>176.66</v>
+      </c>
+      <c r="N10" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="P10" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>Jan 26 (unverified)</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="n"/>
+      <c r="S10" s="12">
+        <f>J10/L10-1</f>
+        <v/>
+      </c>
+      <c r="T10" s="12">
+        <f>J10/K10-1</f>
+        <v/>
+      </c>
+      <c r="U10" s="9">
+        <f>L10*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V10" s="9">
+        <f>L10*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W10" s="9">
+        <f>L10*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X10" s="12">
+        <f>J10/W10-1</f>
+        <v/>
+      </c>
+      <c r="Y10" s="12">
+        <f>IF(N(M10)&gt;0,M10/W10-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z10" s="9">
+        <f>U10</f>
+        <v/>
+      </c>
+      <c r="AA10" s="15">
+        <f>IFERROR(IF(N(M10)&gt;W10,(M10-W10)/(W10-Z10),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB10" s="24">
+        <f>IFERROR(N10/(N10+O10+P10),"")</f>
+        <v/>
+      </c>
+      <c r="AC10" s="16">
+        <f>IF(D10="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R10),Inputs!$B$5&lt;R10,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R10,"m/d"),IF(J10&lt;U10,"BELOW ZONE: wait for 200-day reclaim",IF(J10&gt;V10,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q10),AND(Q10&gt;Inputs!$B$5,Q10-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M10)&lt;=J10,"IN ZONE: analysts see no upside",IF(J10&lt;=W10,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD10" s="17" t="inlineStr">
+        <is>
+          <t>Analyst mean target is BELOW price; 10 Sells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ASML Holding</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -36% (med)</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>1675.7</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>1708.14</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>1595.65</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>2408.5</v>
+      </c>
+      <c r="N11" s="23" t="n">
+        <v>37</v>
+      </c>
+      <c r="O11" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P11" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q11" s="8" t="n">
+        <v>46414</v>
+      </c>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="12">
+        <f>J11/L11-1</f>
+        <v/>
+      </c>
+      <c r="T11" s="12">
+        <f>J11/K11-1</f>
+        <v/>
+      </c>
+      <c r="U11" s="9">
+        <f>L11*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V11" s="9">
+        <f>L11*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W11" s="9">
+        <f>L11*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X11" s="12">
+        <f>J11/W11-1</f>
+        <v/>
+      </c>
+      <c r="Y11" s="12">
+        <f>IF(N(M11)&gt;0,M11/W11-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z11" s="9">
+        <f>U11</f>
+        <v/>
+      </c>
+      <c r="AA11" s="15">
+        <f>IFERROR(IF(N(M11)&gt;W11,(M11-W11)/(W11-Z11),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB11" s="24">
+        <f>IFERROR(N11/(N11+O11+P11),"")</f>
+        <v/>
+      </c>
+      <c r="AC11" s="16">
+        <f>IF(D11="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R11),Inputs!$B$5&lt;R11,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R11,"m/d"),IF(J11&lt;U11,"BELOW ZONE: wait for 200-day reclaim",IF(J11&gt;V11,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q11),AND(Q11&gt;Inputs!$B$5,Q11-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M11)&lt;=J11,"IN ZONE: analysts see no upside",IF(J11&lt;=W11,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD11" s="17" t="inlineStr">
+        <is>
+          <t>Double bottom forming; -3.6% after hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>FNV</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Franco-Nevada</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>FAIR -3% (med)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>231.6</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>252.44</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>240.07</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>287.68</v>
+      </c>
+      <c r="N12" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="O12" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>46337</v>
+      </c>
+      <c r="R12" s="5" t="n"/>
+      <c r="S12" s="12">
+        <f>J12/L12-1</f>
+        <v/>
+      </c>
+      <c r="T12" s="12">
+        <f>J12/K12-1</f>
+        <v/>
+      </c>
+      <c r="U12" s="9">
+        <f>L12*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V12" s="9">
+        <f>L12*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W12" s="9">
+        <f>L12*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X12" s="12">
+        <f>J12/W12-1</f>
+        <v/>
+      </c>
+      <c r="Y12" s="12">
+        <f>IF(N(M12)&gt;0,M12/W12-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z12" s="9">
+        <f>U12</f>
+        <v/>
+      </c>
+      <c r="AA12" s="15">
+        <f>IFERROR(IF(N(M12)&gt;W12,(M12-W12)/(W12-Z12),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB12" s="24">
+        <f>IFERROR(N12/(N12+O12+P12),"")</f>
+        <v/>
+      </c>
+      <c r="AC12" s="16">
+        <f>IF(D12="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R12),Inputs!$B$5&lt;R12,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R12,"m/d"),IF(J12&lt;U12,"BELOW ZONE: wait for 200-day reclaim",IF(J12&gt;V12,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q12),AND(Q12&gt;Inputs!$B$5,Q12-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M12)&lt;=J12,"IN ZONE: analysts see no upside",IF(J12&lt;=W12,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD12" s="17" t="inlineStr">
+        <is>
+          <t>Gold royalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>HOOD</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Robinhood Markets</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>HELD</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>91.59</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>108.69</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>92.76000000000001</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>133.63</v>
+      </c>
+      <c r="N13" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="O13" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="P13" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>Feb 9 (unverified)</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="12">
+        <f>J13/L13-1</f>
+        <v/>
+      </c>
+      <c r="T13" s="12">
+        <f>J13/K13-1</f>
+        <v/>
+      </c>
+      <c r="U13" s="9">
+        <f>L13*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V13" s="9">
+        <f>L13*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W13" s="9">
+        <f>L13*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X13" s="12">
+        <f>J13/W13-1</f>
+        <v/>
+      </c>
+      <c r="Y13" s="12">
+        <f>IF(N(M13)&gt;0,M13/W13-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z13" s="9">
+        <f>U13</f>
+        <v/>
+      </c>
+      <c r="AA13" s="15">
+        <f>IFERROR(IF(N(M13)&gt;W13,(M13-W13)/(W13-Z13),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB13" s="24">
+        <f>IFERROR(N13/(N13+O13+P13),"")</f>
+        <v/>
+      </c>
+      <c r="AC13" s="16">
+        <f>IF(D13="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R13),Inputs!$B$5&lt;R13,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R13,"m/d"),IF(J13&lt;U13,"BELOW ZONE: wait for 200-day reclaim",IF(J13&gt;V13,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q13),AND(Q13&gt;Inputs!$B$5,Q13-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M13)&lt;=J13,"IN ZONE: analysts see no upside",IF(J13&lt;=W13,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD13" s="17" t="inlineStr">
+        <is>
+          <t>Held as a fractional leftover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>NBIX</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Neurocrine Biosciences</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE +100% (low)</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>146.38</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>146.75</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>147.32</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>207.37</v>
+      </c>
+      <c r="N14" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="O14" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P14" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="8" t="n">
+        <v>46328</v>
+      </c>
+      <c r="R14" s="5" t="n"/>
+      <c r="S14" s="12">
+        <f>J14/L14-1</f>
+        <v/>
+      </c>
+      <c r="T14" s="12">
+        <f>J14/K14-1</f>
+        <v/>
+      </c>
+      <c r="U14" s="9">
+        <f>L14*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V14" s="9">
+        <f>L14*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W14" s="9">
+        <f>L14*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X14" s="12">
+        <f>J14/W14-1</f>
+        <v/>
+      </c>
+      <c r="Y14" s="12">
+        <f>IF(N(M14)&gt;0,M14/W14-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z14" s="9">
+        <f>U14</f>
+        <v/>
+      </c>
+      <c r="AA14" s="15">
+        <f>IFERROR(IF(N(M14)&gt;W14,(M14-W14)/(W14-Z14),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB14" s="24">
+        <f>IFERROR(N14/(N14+O14+P14),"")</f>
+        <v/>
+      </c>
+      <c r="AC14" s="16">
+        <f>IF(D14="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R14),Inputs!$B$5&lt;R14,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R14,"m/d"),IF(J14&lt;U14,"BELOW ZONE: wait for 200-day reclaim",IF(J14&gt;V14,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q14),AND(Q14&gt;Inputs!$B$5,Q14-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M14)&lt;=J14,"IN ZONE: analysts see no upside",IF(J14&lt;=W14,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD14" s="17" t="inlineStr">
+        <is>
+          <t>Reports 11/2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>ADBE</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Adobe</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>43 PULLING BACK</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE +100% (low)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>AT RISK</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>248.12</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>254.84</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>250.71</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>269.5</v>
+      </c>
+      <c r="N15" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="O15" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="P15" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>Dec 10 (unverified)</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="n"/>
+      <c r="S15" s="12">
+        <f>J15/L15-1</f>
+        <v/>
+      </c>
+      <c r="T15" s="12">
+        <f>J15/K15-1</f>
+        <v/>
+      </c>
+      <c r="U15" s="9">
+        <f>L15*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V15" s="9">
+        <f>L15*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W15" s="9">
+        <f>L15*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X15" s="12">
+        <f>J15/W15-1</f>
+        <v/>
+      </c>
+      <c r="Y15" s="12">
+        <f>IF(N(M15)&gt;0,M15/W15-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z15" s="9">
+        <f>U15</f>
+        <v/>
+      </c>
+      <c r="AA15" s="15">
+        <f>IFERROR(IF(N(M15)&gt;W15,(M15-W15)/(W15-Z15),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB15" s="24">
+        <f>IFERROR(N15/(N15+O15+P15),"")</f>
+        <v/>
+      </c>
+      <c r="AC15" s="16">
+        <f>IF(D15="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R15),Inputs!$B$5&lt;R15,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R15,"m/d"),IF(J15&lt;U15,"BELOW ZONE: wait for 200-day reclaim",IF(J15&gt;V15,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q15),AND(Q15&gt;Inputs!$B$5,Q15-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M15)&lt;=J15,"IN ZONE: analysts see no upside",IF(J15&lt;=W15,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD15" s="17" t="inlineStr">
+        <is>
+          <t>VALUE TRAP? flag: AI design tools pressure; thesis weakened 10/23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>HELD</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>29 MIXED</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>RICH -14% (low)</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>624.52</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>668.6</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>632.11</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>850.51</v>
+      </c>
+      <c r="N16" s="23" t="n">
+        <v>65</v>
+      </c>
+      <c r="O16" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="P16" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>Jan 27 (unverified)</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="n"/>
+      <c r="S16" s="12">
+        <f>J16/L16-1</f>
+        <v/>
+      </c>
+      <c r="T16" s="12">
+        <f>J16/K16-1</f>
+        <v/>
+      </c>
+      <c r="U16" s="9">
+        <f>L16*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V16" s="9">
+        <f>L16*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W16" s="9">
+        <f>L16*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X16" s="12">
+        <f>J16/W16-1</f>
+        <v/>
+      </c>
+      <c r="Y16" s="12">
+        <f>IF(N(M16)&gt;0,M16/W16-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z16" s="9">
+        <f>U16</f>
+        <v/>
+      </c>
+      <c r="AA16" s="15">
+        <f>IFERROR(IF(N(M16)&gt;W16,(M16-W16)/(W16-Z16),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB16" s="24">
+        <f>IFERROR(N16/(N16+O16+P16),"")</f>
+        <v/>
+      </c>
+      <c r="AC16" s="16">
+        <f>IF(D16="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R16),Inputs!$B$5&lt;R16,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R16,"m/d"),IF(J16&lt;U16,"BELOW ZONE: wait for 200-day reclaim",IF(J16&gt;V16,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q16),AND(Q16&gt;Inputs!$B$5,Q16-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M16)&lt;=J16,"IN ZONE: analysts see no upside",IF(J16&lt;=W16,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD16" s="17" t="inlineStr">
+        <is>
+          <t>Already held (~15% of the joint account).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>NEM</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Newmont</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>29 MIXED</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -28% (low)</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>112.49</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>137.61</v>
+      </c>
+      <c r="N17" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="O17" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P17" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Feb 19 (unverified)</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="12">
+        <f>J17/L17-1</f>
+        <v/>
+      </c>
+      <c r="T17" s="12">
+        <f>J17/K17-1</f>
+        <v/>
+      </c>
+      <c r="U17" s="9">
+        <f>L17*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V17" s="9">
+        <f>L17*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W17" s="9">
+        <f>L17*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X17" s="12">
+        <f>J17/W17-1</f>
+        <v/>
+      </c>
+      <c r="Y17" s="12">
+        <f>IF(N(M17)&gt;0,M17/W17-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z17" s="9">
+        <f>U17</f>
+        <v/>
+      </c>
+      <c r="AA17" s="15">
+        <f>IFERROR(IF(N(M17)&gt;W17,(M17-W17)/(W17-Z17),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB17" s="24">
+        <f>IFERROR(N17/(N17+O17+P17),"")</f>
+        <v/>
+      </c>
+      <c r="AC17" s="16">
+        <f>IF(D17="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R17),Inputs!$B$5&lt;R17,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R17,"m/d"),IF(J17&lt;U17,"BELOW ZONE: wait for 200-day reclaim",IF(J17&gt;V17,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q17),AND(Q17&gt;Inputs!$B$5,Q17-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M17)&lt;=J17,"IN ZONE: analysts see no upside",IF(J17&lt;=W17,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD17" s="17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Applied Materials</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>29 MIXED</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -50% (low)</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>INNOVATING</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>421.66</v>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>459.67</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>444.04</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>651.64</v>
+      </c>
+      <c r="N18" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="O18" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="P18" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="8" t="n">
+        <v>46338</v>
+      </c>
+      <c r="R18" s="5" t="n"/>
+      <c r="S18" s="12">
+        <f>J18/L18-1</f>
+        <v/>
+      </c>
+      <c r="T18" s="12">
+        <f>J18/K18-1</f>
+        <v/>
+      </c>
+      <c r="U18" s="9">
+        <f>L18*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V18" s="9">
+        <f>L18*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W18" s="9">
+        <f>L18*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X18" s="12">
+        <f>J18/W18-1</f>
+        <v/>
+      </c>
+      <c r="Y18" s="12">
+        <f>IF(N(M18)&gt;0,M18/W18-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z18" s="9">
+        <f>U18</f>
+        <v/>
+      </c>
+      <c r="AA18" s="15">
+        <f>IFERROR(IF(N(M18)&gt;W18,(M18-W18)/(W18-Z18),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB18" s="24">
+        <f>IFERROR(N18/(N18+O18+P18),"")</f>
+        <v/>
+      </c>
+      <c r="AC18" s="16">
+        <f>IF(D18="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R18),Inputs!$B$5&lt;R18,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R18,"m/d"),IF(J18&lt;U18,"BELOW ZONE: wait for 200-day reclaim",IF(J18&gt;V18,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q18),AND(Q18&gt;Inputs!$B$5,Q18-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M18)&lt;=J18,"IN ZONE: analysts see no upside",IF(J18&lt;=W18,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD18" s="17" t="inlineStr">
+        <is>
+          <t>-4.5% after hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>RGLD</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Royal Gold</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>14 EXTENDED</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>FAIR +3% (high)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>236.83</v>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>246.65</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>241.42</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>310.08</v>
+      </c>
+      <c r="N19" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="O19" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="P19" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="8" t="inlineStr">
+        <is>
+          <t>Nov 5 (unverified)</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="n"/>
+      <c r="S19" s="12">
+        <f>J19/L19-1</f>
+        <v/>
+      </c>
+      <c r="T19" s="12">
+        <f>J19/K19-1</f>
+        <v/>
+      </c>
+      <c r="U19" s="9">
+        <f>L19*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V19" s="9">
+        <f>L19*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W19" s="9">
+        <f>L19*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X19" s="12">
+        <f>J19/W19-1</f>
+        <v/>
+      </c>
+      <c r="Y19" s="12">
+        <f>IF(N(M19)&gt;0,M19/W19-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z19" s="9">
+        <f>U19</f>
+        <v/>
+      </c>
+      <c r="AA19" s="15">
+        <f>IFERROR(IF(N(M19)&gt;W19,(M19-W19)/(W19-Z19),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB19" s="24">
+        <f>IFERROR(N19/(N19+O19+P19),"")</f>
+        <v/>
+      </c>
+      <c r="AC19" s="16">
+        <f>IF(D19="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R19),Inputs!$B$5&lt;R19,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R19,"m/d"),IF(J19&lt;U19,"BELOW ZONE: wait for 200-day reclaim",IF(J19&gt;V19,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q19),AND(Q19&gt;Inputs!$B$5,Q19-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M19)&lt;=J19,"IN ZONE: analysts see no upside",IF(J19&lt;=W19,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD19" s="17" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Western Digital</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>14 EXTENDED</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -50% (low)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>395.41</v>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>423.52</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>418.23</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>621.78</v>
+      </c>
+      <c r="N20" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="O20" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="P20" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>Jan 28 (unverified)</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="n"/>
+      <c r="S20" s="12">
+        <f>J20/L20-1</f>
+        <v/>
+      </c>
+      <c r="T20" s="12">
+        <f>J20/K20-1</f>
+        <v/>
+      </c>
+      <c r="U20" s="9">
+        <f>L20*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V20" s="9">
+        <f>L20*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W20" s="9">
+        <f>L20*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X20" s="12">
+        <f>J20/W20-1</f>
+        <v/>
+      </c>
+      <c r="Y20" s="12">
+        <f>IF(N(M20)&gt;0,M20/W20-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z20" s="9">
+        <f>U20</f>
+        <v/>
+      </c>
+      <c r="AA20" s="15">
+        <f>IFERROR(IF(N(M20)&gt;W20,(M20-W20)/(W20-Z20),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB20" s="24">
+        <f>IFERROR(N20/(N20+O20+P20),"")</f>
+        <v/>
+      </c>
+      <c r="AC20" s="16">
+        <f>IF(D20="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R20),Inputs!$B$5&lt;R20,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R20,"m/d"),IF(J20&lt;U20,"BELOW ZONE: wait for 200-day reclaim",IF(J20&gt;V20,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q20),AND(Q20&gt;Inputs!$B$5,Q20-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M20)&lt;=J20,"IN ZONE: analysts see no upside",IF(J20&lt;=W20,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD20" s="17" t="inlineStr">
+        <is>
+          <t>-4.5% after hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>PAC</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Aeroportuario del Pacifico</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>0 EXTENDED</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE +58% (med)</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>227.47</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>208.31</v>
+      </c>
+      <c r="L21" s="7" t="n">
+        <v>236.65</v>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="N21" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="O21" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="P21" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t>Feb 22 (unverified)</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="n"/>
+      <c r="S21" s="12">
+        <f>J21/L21-1</f>
+        <v/>
+      </c>
+      <c r="T21" s="12">
+        <f>J21/K21-1</f>
+        <v/>
+      </c>
+      <c r="U21" s="9">
+        <f>L21*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V21" s="9">
+        <f>L21*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W21" s="9">
+        <f>L21*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X21" s="12">
+        <f>J21/W21-1</f>
+        <v/>
+      </c>
+      <c r="Y21" s="12">
+        <f>IF(N(M21)&gt;0,M21/W21-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z21" s="9">
+        <f>U21</f>
+        <v/>
+      </c>
+      <c r="AA21" s="15">
+        <f>IFERROR(IF(N(M21)&gt;W21,(M21-W21)/(W21-Z21),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB21" s="24">
+        <f>IFERROR(N21/(N21+O21+P21),"")</f>
+        <v/>
+      </c>
+      <c r="AC21" s="16">
+        <f>IF(D21="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R21),Inputs!$B$5&lt;R21,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R21,"m/d"),IF(J21&lt;U21,"BELOW ZONE: wait for 200-day reclaim",IF(J21&gt;V21,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q21),AND(Q21&gt;Inputs!$B$5,Q21-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M21)&lt;=J21,"IN ZONE: analysts see no upside",IF(J21&lt;=W21,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD21" s="17" t="inlineStr">
+        <is>
+          <t>Analyst target last updated 2020: stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Cadence Design</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>HELD</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>0 EXTENDED</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>RICH -13% (med)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>342.75</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>320.24</v>
+      </c>
+      <c r="L22" s="7" t="n">
+        <v>327.46</v>
+      </c>
+      <c r="M22" s="7" t="n">
+        <v>415.04</v>
+      </c>
+      <c r="N22" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="O22" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="P22" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="8" t="inlineStr">
+        <is>
+          <t>Feb 17 (unverified)</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="n"/>
+      <c r="S22" s="12">
+        <f>J22/L22-1</f>
+        <v/>
+      </c>
+      <c r="T22" s="12">
+        <f>J22/K22-1</f>
+        <v/>
+      </c>
+      <c r="U22" s="9">
+        <f>L22*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V22" s="9">
+        <f>L22*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W22" s="9">
+        <f>L22*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X22" s="12">
+        <f>J22/W22-1</f>
+        <v/>
+      </c>
+      <c r="Y22" s="12">
+        <f>IF(N(M22)&gt;0,M22/W22-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z22" s="9">
+        <f>U22</f>
+        <v/>
+      </c>
+      <c r="AA22" s="15">
+        <f>IFERROR(IF(N(M22)&gt;W22,(M22-W22)/(W22-Z22),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB22" s="24">
+        <f>IFERROR(N22/(N22+O22+P22),"")</f>
+        <v/>
+      </c>
+      <c r="AC22" s="16">
+        <f>IF(D22="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R22),Inputs!$B$5&lt;R22,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R22,"m/d"),IF(J22&lt;U22,"BELOW ZONE: wait for 200-day reclaim",IF(J22&gt;V22,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q22),AND(Q22&gt;Inputs!$B$5,Q22-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M22)&lt;=J22,"IN ZONE: analysts see no upside",IF(J22&lt;=W22,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD22" s="17" t="inlineStr">
+        <is>
+          <t>Already held (20 sh).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>ISRG</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Intuitive Surgical</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>0 EXTENDED</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE +43% (high)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>AT RISK</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>448.76</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>400.3</v>
+      </c>
+      <c r="L23" s="7" t="n">
+        <v>433.61</v>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>489.57</v>
+      </c>
+      <c r="N23" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="O23" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="P23" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q23" s="8" t="inlineStr">
+        <is>
+          <t>Jan 22 (unverified)</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="n"/>
+      <c r="S23" s="12">
+        <f>J23/L23-1</f>
+        <v/>
+      </c>
+      <c r="T23" s="12">
+        <f>J23/K23-1</f>
+        <v/>
+      </c>
+      <c r="U23" s="9">
+        <f>L23*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V23" s="9">
+        <f>L23*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W23" s="9">
+        <f>L23*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X23" s="12">
+        <f>J23/W23-1</f>
+        <v/>
+      </c>
+      <c r="Y23" s="12">
+        <f>IF(N(M23)&gt;0,M23/W23-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z23" s="9">
+        <f>U23</f>
+        <v/>
+      </c>
+      <c r="AA23" s="15">
+        <f>IFERROR(IF(N(M23)&gt;W23,(M23-W23)/(W23-Z23),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB23" s="24">
+        <f>IFERROR(N23/(N23+O23+P23),"")</f>
+        <v/>
+      </c>
+      <c r="AC23" s="16">
+        <f>IF(D23="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R23),Inputs!$B$5&lt;R23,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R23,"m/d"),IF(J23&lt;U23,"BELOW ZONE: wait for 200-day reclaim",IF(J23&gt;V23,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q23),AND(Q23&gt;Inputs!$B$5,Q23-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M23)&lt;=J23,"IN ZONE: analysts see no upside",IF(J23&lt;=W23,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD23" s="17" t="inlineStr">
+        <is>
+          <t>VALUE TRAP? flag from the quant grade; research says innovating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>TROW</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>T. Rowe Price</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>0 EXTENDED</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE +40% (med)</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>AT RISK</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>106.63</v>
+      </c>
+      <c r="K24" s="7" t="n">
+        <v>105.77</v>
+      </c>
+      <c r="L24" s="7" t="n">
+        <v>103.68</v>
+      </c>
+      <c r="M24" s="7" t="n">
+        <v>102.83</v>
+      </c>
+      <c r="N24" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="P24" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q24" s="8" t="inlineStr">
+        <is>
+          <t>Reported 10/29</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="n"/>
+      <c r="S24" s="12">
+        <f>J24/L24-1</f>
+        <v/>
+      </c>
+      <c r="T24" s="12">
+        <f>J24/K24-1</f>
+        <v/>
+      </c>
+      <c r="U24" s="9">
+        <f>L24*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V24" s="9">
+        <f>L24*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W24" s="9">
+        <f>L24*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X24" s="12">
+        <f>J24/W24-1</f>
+        <v/>
+      </c>
+      <c r="Y24" s="12">
+        <f>IF(N(M24)&gt;0,M24/W24-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z24" s="9">
+        <f>U24</f>
+        <v/>
+      </c>
+      <c r="AA24" s="15">
+        <f>IFERROR(IF(N(M24)&gt;W24,(M24-W24)/(W24-Z24),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB24" s="24">
+        <f>IFERROR(N24/(N24+O24+P24),"")</f>
+        <v/>
+      </c>
+      <c r="AC24" s="16">
+        <f>IF(D24="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R24),Inputs!$B$5&lt;R24,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R24,"m/d"),IF(J24&lt;U24,"BELOW ZONE: wait for 200-day reclaim",IF(J24&gt;V24,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q24),AND(Q24&gt;Inputs!$B$5,Q24-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M24)&lt;=J24,"IN ZONE: analysts see no upside",IF(J24&lt;=W24,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD24" s="17" t="inlineStr">
+        <is>
+          <t>VALUE TRAP? Losing assets to passive funds. No Buy ratings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>SKHY</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>SK hynix (ADR)</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE +100% (low)</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>162.09</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>169.17</v>
+      </c>
+      <c r="L25" s="7" t="n">
+        <v>154.83</v>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>263.91</v>
+      </c>
+      <c r="N25" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="O25" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P25" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="8" t="inlineStr">
+        <is>
+          <t>Feb 13 (unverified)</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="n"/>
+      <c r="S25" s="12">
+        <f>J25/L25-1</f>
+        <v/>
+      </c>
+      <c r="T25" s="12">
+        <f>J25/K25-1</f>
+        <v/>
+      </c>
+      <c r="U25" s="9">
+        <f>L25*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V25" s="9">
+        <f>L25*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W25" s="9">
+        <f>L25*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X25" s="12">
+        <f>J25/W25-1</f>
+        <v/>
+      </c>
+      <c r="Y25" s="12">
+        <f>IF(N(M25)&gt;0,M25/W25-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z25" s="9">
+        <f>U25</f>
+        <v/>
+      </c>
+      <c r="AA25" s="15">
+        <f>IFERROR(IF(N(M25)&gt;W25,(M25-W25)/(W25-Z25),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB25" s="24">
+        <f>IFERROR(N25/(N25+O25+P25),"")</f>
+        <v/>
+      </c>
+      <c r="AC25" s="16">
+        <f>IF(D25="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R25),Inputs!$B$5&lt;R25,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R25,"m/d"),IF(J25&lt;U25,"BELOW ZONE: wait for 200-day reclaim",IF(J25&gt;V25,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q25),AND(Q25&gt;Inputs!$B$5,Q25-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M25)&lt;=J25,"IN ZONE: analysts see no upside",IF(J25&lt;=W25,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD25" s="17" t="inlineStr">
+        <is>
+          <t>-5.3% after hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>PSA</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Public Storage</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>317.06</v>
+      </c>
+      <c r="K26" s="7" t="n">
+        <v>298.61</v>
+      </c>
+      <c r="L26" s="7" t="n">
+        <v>302.64</v>
+      </c>
+      <c r="M26" s="7" t="n">
+        <v>330.06</v>
+      </c>
+      <c r="N26" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="O26" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="P26" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="8" t="inlineStr">
+        <is>
+          <t>Feb 11 (unverified)</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="n"/>
+      <c r="S26" s="12">
+        <f>J26/L26-1</f>
+        <v/>
+      </c>
+      <c r="T26" s="12">
+        <f>J26/K26-1</f>
+        <v/>
+      </c>
+      <c r="U26" s="9">
+        <f>L26*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V26" s="9">
+        <f>L26*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W26" s="9">
+        <f>L26*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X26" s="12">
+        <f>J26/W26-1</f>
+        <v/>
+      </c>
+      <c r="Y26" s="12">
+        <f>IF(N(M26)&gt;0,M26/W26-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z26" s="9">
+        <f>U26</f>
+        <v/>
+      </c>
+      <c r="AA26" s="15">
+        <f>IFERROR(IF(N(M26)&gt;W26,(M26-W26)/(W26-Z26),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB26" s="24">
+        <f>IFERROR(N26/(N26+O26+P26),"")</f>
+        <v/>
+      </c>
+      <c r="AC26" s="16">
+        <f>IF(D26="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R26),Inputs!$B$5&lt;R26,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R26,"m/d"),IF(J26&lt;U26,"BELOW ZONE: wait for 200-day reclaim",IF(J26&gt;V26,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q26),AND(Q26&gt;Inputs!$B$5,Q26-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M26)&lt;=J26,"IN ZONE: analysts see no upside",IF(J26&lt;=W26,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD26" s="17" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>KEYS</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Keysight</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Buy Zone</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="n">
+        <v>23</v>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -40% (med)</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>329.84</v>
+      </c>
+      <c r="K27" s="7" t="n">
+        <v>341.12</v>
+      </c>
+      <c r="L27" s="7" t="n">
+        <v>316.26</v>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>424.18</v>
+      </c>
+      <c r="N27" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="O27" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="P27" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="8" t="n">
+        <v>46345</v>
+      </c>
+      <c r="R27" s="5" t="n"/>
+      <c r="S27" s="12">
+        <f>J27/L27-1</f>
+        <v/>
+      </c>
+      <c r="T27" s="12">
+        <f>J27/K27-1</f>
+        <v/>
+      </c>
+      <c r="U27" s="9">
+        <f>L27*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V27" s="9">
+        <f>L27*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W27" s="9">
+        <f>L27*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X27" s="12">
+        <f>J27/W27-1</f>
+        <v/>
+      </c>
+      <c r="Y27" s="12">
+        <f>IF(N(M27)&gt;0,M27/W27-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z27" s="9">
+        <f>U27</f>
+        <v/>
+      </c>
+      <c r="AA27" s="15">
+        <f>IFERROR(IF(N(M27)&gt;W27,(M27-W27)/(W27-Z27),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB27" s="24">
+        <f>IFERROR(N27/(N27+O27+P27),"")</f>
+        <v/>
+      </c>
+      <c r="AC27" s="16">
+        <f>IF(D27="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R27),Inputs!$B$5&lt;R27,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R27,"m/d"),IF(J27&lt;U27,"BELOW ZONE: wait for 200-day reclaim",IF(J27&gt;V27,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q27),AND(Q27&gt;Inputs!$B$5,Q27-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M27)&lt;=J27,"IN ZONE: analysts see no upside",IF(J27&lt;=W27,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD27" s="17" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>MOD</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Modine Manufacturing</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Re-buy</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>WAIT (re-buy stage)</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>138.79</v>
+      </c>
+      <c r="K28" s="7" t="n">
+        <v>175.88</v>
+      </c>
+      <c r="L28" s="7" t="n">
+        <v>216.14</v>
+      </c>
+      <c r="M28" s="7" t="n">
+        <v>282.48</v>
+      </c>
+      <c r="N28" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="O28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="8" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="R28" s="8" t="n">
+        <v>46340</v>
+      </c>
+      <c r="S28" s="12">
+        <f>J28/L28-1</f>
+        <v/>
+      </c>
+      <c r="T28" s="12">
+        <f>J28/K28-1</f>
+        <v/>
+      </c>
+      <c r="U28" s="9">
+        <f>L28*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V28" s="9">
+        <f>L28*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W28" s="9">
+        <f>L28*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X28" s="12">
+        <f>J28/W28-1</f>
+        <v/>
+      </c>
+      <c r="Y28" s="12">
+        <f>IF(N(M28)&gt;0,M28/W28-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z28" s="9">
+        <f>U28</f>
+        <v/>
+      </c>
+      <c r="AA28" s="15">
+        <f>IFERROR(IF(N(M28)&gt;W28,(M28-W28)/(W28-Z28),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB28" s="24">
+        <f>IFERROR(N28/(N28+O28+P28),"")</f>
+        <v/>
+      </c>
+      <c r="AC28" s="16">
+        <f>IF(D28="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R28),Inputs!$B$5&lt;R28,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R28,"m/d"),IF(J28&lt;U28,"BELOW ZONE: wait for 200-day reclaim",IF(J28&gt;V28,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q28),AND(Q28&gt;Inputs!$B$5,Q28-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M28)&lt;=J28,"IN ZONE: analysts see no upside",IF(J28&lt;=W28,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD28" s="17" t="inlineStr">
+        <is>
+          <t>Sold 10/14 @ 162.10 at a loss: do not rebuy before the wash-sale date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>COUNT</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="n"/>
+      <c r="C30" s="18" t="n"/>
+      <c r="D30" s="18" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="F30" s="18" t="n"/>
+      <c r="G30" s="18" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="18" t="n"/>
+      <c r="J30" s="18" t="n"/>
+      <c r="K30" s="18" t="n"/>
+      <c r="L30" s="18" t="n"/>
+      <c r="M30" s="18" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
+      <c r="P30" s="18" t="n"/>
+      <c r="Q30" s="18" t="n"/>
+      <c r="R30" s="18" t="n"/>
+      <c r="S30" s="18" t="n"/>
+      <c r="T30" s="18" t="n"/>
+      <c r="U30" s="18" t="n"/>
+      <c r="V30" s="18" t="n"/>
+      <c r="W30" s="18" t="n"/>
+      <c r="X30" s="18" t="n"/>
+      <c r="Y30" s="18" t="n"/>
+      <c r="Z30" s="18" t="n"/>
+      <c r="AA30" s="18" t="n"/>
+      <c r="AB30" s="18" t="n"/>
+      <c r="AC30" s="18">
+        <f>COUNTIF(AC5:AC28,"IN ZONE*")&amp;" in zone, "&amp;COUNTIF(AC5:AC28,"BELOW*")&amp;" below, "&amp;COUNTIF(AC5:AC28,"ABOVE*")&amp;" above"</f>
+        <v/>
+      </c>
+      <c r="AD30" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:AD28"/>
+  <conditionalFormatting sqref="AC5:AC28">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>LEFT(AC5,7)="IN ZONE"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>OR(LEFT(AC5,4)="WASH",ISNUMBER(SEARCH("earnings",AC5)),ISNUMBER(SEARCH("no upside",AC5)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>LEFT(AC5,5)="BELOW"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I28">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"AT RISK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4199,17 +7258,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>Assumption</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>What it does</t>
         </is>
@@ -4253,7 +7312,7 @@
           <t>Trim 1 trigger (% of final target)</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="26" t="n">
         <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -4268,7 +7327,7 @@
           <t>Trim 2 stretch above target</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="26" t="n">
         <v>0.15</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -4283,7 +7342,7 @@
           <t>Shares sold at each trim</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="26" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -4298,7 +7357,7 @@
           <t>Support buffer below 60-day low</t>
         </is>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="27" t="n">
         <v>0.01</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -4313,7 +7372,7 @@
           <t>Max loss from cost - stocks</t>
         </is>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="26" t="n">
         <v>0.25</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -4328,7 +7387,7 @@
           <t>Max loss from cost - leveraged ETFs</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="26" t="n">
         <v>0.3</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -4343,7 +7402,7 @@
           <t>Trailing stop %</t>
         </is>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="26" t="n">
         <v>0.15</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -4358,7 +7417,7 @@
           <t>Position cap - stocks (% of portfolio)</t>
         </is>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="26" t="n">
         <v>0.15</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -4373,7 +7432,7 @@
           <t>Position cap - leveraged ETFs</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="26" t="n">
         <v>0.05</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -4388,12 +7447,57 @@
           <t>Earnings warning window (days)</t>
         </is>
       </c>
-      <c r="B16" s="26" t="n">
+      <c r="B16" s="23" t="n">
         <v>7</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>Flags a holding reporting within this many days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Watchlist: buy zone low vs 200-day</t>
+        </is>
+      </c>
+      <c r="B17" s="26" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Bottom of the buy zone. Below it the 200-day has failed: wait for a reclaim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Watchlist: buy zone high vs 200-day</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Top of the buy zone. Above it the name is extended: wait.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Watchlist: entry vs 200-day</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Buy target = 200-day SMA x (1 + this). 0% = buy at the line.</t>
         </is>
       </c>
     </row>
@@ -4407,20 +7511,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>How the numbers are set</t>
         </is>
@@ -4504,65 +7608,100 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WATCHLIST (Watchlist sheet): the Quality @ 200-day routine's buy-zone names (business grade &gt;= 7/8, near the 200-day),</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
-        <is>
-          <t>Sources</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ranked by pre-breakout chart setup (most pulled back first), plus the re-buy watch (MOD).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Positions, quotes, 50/200-day SMA, 60-day range, 52-wk high, earnings dates: Robinhood (pulled 2026-10-30).</t>
+          <t xml:space="preserve">  BUY TARGET = 200-day SMA x (1 + entry offset). BUY ZONE = 200-day -8% to +5%. Below the zone = trend failed, wait for a reclaim.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Targets: joint_price_targets.json (2026-10-29). Valuation and disruption grades: valuation.json (2026-10-28/29).</t>
+          <t xml:space="preserve">  WATCH REVIEW LEVEL = bottom of the buy zone: where a new buy is wrong. UPSIDE / REWARD:RISK are measured from the buy target to the analyst mean target.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STATUS is a prompt to research, not a buy order: every name still needs a news/thesis check and a wash-sale check before buying.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
-        <is>
-          <t>Not included</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>EPIX^ (25 sh, $0 cost) has no quote: likely a delisted or escrowed position. Check it in the app.</t>
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>Sources</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Positions, quotes, 50/200-day SMA, 60-day range, 52-wk high, earnings dates: Robinhood (pulled 2026-10-30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Targets: joint_price_targets.json (2026-10-29). Valuation and disruption grades: valuation.json (2026-10-28/29).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Not included</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EPIX^ (25 sh, $0 cost) has no quote: likely a delisted or escrowed position. Check it in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Taxes: this is a taxable account. Check wash-sale lockouts (Robinhood list 'Wash-Sale Lockout') before selling at a loss and rebuying.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="27" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
         <is>
           <t>Refresh</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Edit the blue cells, or update SNAPSHOT in build_joint_tracker.py and re-run it.</t>
         </is>

</xml_diff>

<commit_message>
Joint tracker: add 10 new-industry quality names to the Watchlist
Payments (MA, CPAY, AFRM), biotech (VRTX, INCY), rail (UNP), staples (MNST),
REIT (SPG), consumer tech (AAPL), networking (ANET). Each scores >= 7/8 on the
quality watch's business test; found by a 5-20%-above-200-day screen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XBawetM5mpZm52AQxpa6eR
</commit_message>
<xml_diff>
--- a/joint_portfolio_tracker.xlsx
+++ b/joint_portfolio_tracker.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Holdings'!$A$5:$AP$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Watchlist'!$A$4:$AD$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Watchlist'!$A$4:$AD$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4179,12 +4179,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD30"/>
+  <dimension ref="A1:AD40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -4217,7 +4217,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Joint Watchlist - Quality @ 200-day Buy Zone + Re-buy Watch</t>
+          <t>Joint Watchlist - Quality @ 200-day Buy Zone, Re-buy Watch, New Industries</t>
         </is>
       </c>
     </row>
@@ -7168,48 +7168,1186 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>SPG</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Simon Property Group</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Malls REIT</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>FAIR -2% (high)</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="n">
+        <v>215.72</v>
+      </c>
+      <c r="K29" s="7" t="n">
+        <v>207.18</v>
+      </c>
+      <c r="L29" s="7" t="n">
+        <v>205.72</v>
+      </c>
+      <c r="M29" s="7" t="n">
+        <v>228.89</v>
+      </c>
+      <c r="N29" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="O29" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="P29" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="8" t="n">
+        <v>46331</v>
+      </c>
+      <c r="R29" s="5" t="n"/>
+      <c r="S29" s="12">
+        <f>J29/L29-1</f>
+        <v/>
+      </c>
+      <c r="T29" s="12">
+        <f>J29/K29-1</f>
+        <v/>
+      </c>
+      <c r="U29" s="9">
+        <f>L29*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V29" s="9">
+        <f>L29*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W29" s="9">
+        <f>L29*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X29" s="12">
+        <f>J29/W29-1</f>
+        <v/>
+      </c>
+      <c r="Y29" s="12">
+        <f>IF(N(M29)&gt;0,M29/W29-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z29" s="9">
+        <f>U29</f>
+        <v/>
+      </c>
+      <c r="AA29" s="15">
+        <f>IFERROR(IF(N(M29)&gt;W29,(M29-W29)/(W29-Z29),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB29" s="24">
+        <f>IFERROR(N29/(N29+O29+P29),"")</f>
+        <v/>
+      </c>
+      <c r="AC29" s="16">
+        <f>IF(D29="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R29),Inputs!$B$5&lt;R29,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R29,"m/d"),IF(J29&lt;U29,"BELOW ZONE: wait for 200-day reclaim",IF(J29&gt;V29,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q29),AND(Q29&gt;Inputs!$B$5,Q29-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M29)&lt;=J29,"IN ZONE: analysts see no upside",IF(J29&lt;=W29,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD29" s="17" t="inlineStr">
+        <is>
+          <t>Only new name already inside the buy zone. Analysts mostly Hold.</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>MNST</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Monster Beverage</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Consumer staples</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>RICH -11% (med)</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>46.35</v>
+      </c>
+      <c r="K30" s="7" t="n">
+        <v>44.75</v>
+      </c>
+      <c r="L30" s="7" t="n">
+        <v>43.04</v>
+      </c>
+      <c r="M30" s="7" t="n">
+        <v>50.69</v>
+      </c>
+      <c r="N30" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="O30" s="23" t="n">
+        <v>13</v>
+      </c>
+      <c r="P30" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="8" t="n">
+        <v>46331</v>
+      </c>
+      <c r="R30" s="5" t="n"/>
+      <c r="S30" s="12">
+        <f>J30/L30-1</f>
+        <v/>
+      </c>
+      <c r="T30" s="12">
+        <f>J30/K30-1</f>
+        <v/>
+      </c>
+      <c r="U30" s="9">
+        <f>L30*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V30" s="9">
+        <f>L30*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W30" s="9">
+        <f>L30*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X30" s="12">
+        <f>J30/W30-1</f>
+        <v/>
+      </c>
+      <c r="Y30" s="12">
+        <f>IF(N(M30)&gt;0,M30/W30-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z30" s="9">
+        <f>U30</f>
+        <v/>
+      </c>
+      <c r="AA30" s="15">
+        <f>IFERROR(IF(N(M30)&gt;W30,(M30-W30)/(W30-Z30),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB30" s="24">
+        <f>IFERROR(N30/(N30+O30+P30),"")</f>
+        <v/>
+      </c>
+      <c r="AC30" s="16">
+        <f>IF(D30="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R30),Inputs!$B$5&lt;R30,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R30,"m/d"),IF(J30&lt;U30,"BELOW ZONE: wait for 200-day reclaim",IF(J30&gt;V30,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q30),AND(Q30&gt;Inputs!$B$5,Q30-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M30)&lt;=J30,"IN ZONE: analysts see no upside",IF(J30&lt;=W30,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD30" s="17" t="inlineStr">
+        <is>
+          <t>Rev +20%, net margin 23%. 2-for-1 split Aug 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>INCY</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Incyte</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Biotech</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>DEEP VALUE (low conf.)</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>INNOVATING</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>120.62</v>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>107.99</v>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>132.78</v>
+      </c>
+      <c r="N31" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="O31" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="P31" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q31" s="8" t="inlineStr">
+        <is>
+          <t>Reported 10/29</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="n"/>
+      <c r="S31" s="12">
+        <f>J31/L31-1</f>
+        <v/>
+      </c>
+      <c r="T31" s="12">
+        <f>J31/K31-1</f>
+        <v/>
+      </c>
+      <c r="U31" s="9">
+        <f>L31*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V31" s="9">
+        <f>L31*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W31" s="9">
+        <f>L31*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X31" s="12">
+        <f>J31/W31-1</f>
+        <v/>
+      </c>
+      <c r="Y31" s="12">
+        <f>IF(N(M31)&gt;0,M31/W31-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z31" s="9">
+        <f>U31</f>
+        <v/>
+      </c>
+      <c r="AA31" s="15">
+        <f>IFERROR(IF(N(M31)&gt;W31,(M31-W31)/(W31-Z31),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB31" s="24">
+        <f>IFERROR(N31/(N31+O31+P31),"")</f>
+        <v/>
+      </c>
+      <c r="AC31" s="16">
+        <f>IF(D31="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R31),Inputs!$B$5&lt;R31,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R31,"m/d"),IF(J31&lt;U31,"BELOW ZONE: wait for 200-day reclaim",IF(J31&gt;V31,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q31),AND(Q31&gt;Inputs!$B$5,Q31-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M31)&lt;=J31,"IN ZONE: analysts see no upside",IF(J31&lt;=W31,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD31" s="17" t="inlineStr">
+        <is>
+          <t>Q3 GAAP loss -$3.86/sh from a one-time $1.23B Vega IPR&amp;D charge; revenue +14%. Analysts split Buy/Hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Arista Networks</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>AI networking</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -32% (low)</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>INNOVATING</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>184.22</v>
+      </c>
+      <c r="K32" s="7" t="n">
+        <v>195.57</v>
+      </c>
+      <c r="L32" s="7" t="n">
+        <v>164.96</v>
+      </c>
+      <c r="M32" s="7" t="n">
+        <v>248.54</v>
+      </c>
+      <c r="N32" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="O32" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="8" t="n">
+        <v>46329</v>
+      </c>
+      <c r="R32" s="5" t="n"/>
+      <c r="S32" s="12">
+        <f>J32/L32-1</f>
+        <v/>
+      </c>
+      <c r="T32" s="12">
+        <f>J32/K32-1</f>
+        <v/>
+      </c>
+      <c r="U32" s="9">
+        <f>L32*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V32" s="9">
+        <f>L32*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W32" s="9">
+        <f>L32*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X32" s="12">
+        <f>J32/W32-1</f>
+        <v/>
+      </c>
+      <c r="Y32" s="12">
+        <f>IF(N(M32)&gt;0,M32/W32-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z32" s="9">
+        <f>U32</f>
+        <v/>
+      </c>
+      <c r="AA32" s="15">
+        <f>IFERROR(IF(N(M32)&gt;W32,(M32-W32)/(W32-Z32),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB32" s="24">
+        <f>IFERROR(N32/(N32+O32+P32),"")</f>
+        <v/>
+      </c>
+      <c r="AC32" s="16">
+        <f>IF(D32="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R32),Inputs!$B$5&lt;R32,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R32,"m/d"),IF(J32&lt;U32,"BELOW ZONE: wait for 200-day reclaim",IF(J32&gt;V32,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q32),AND(Q32&gt;Inputs!$B$5,Q32-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M32)&lt;=J32,"IN ZONE: analysts see no upside",IF(J32&lt;=W32,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD32" s="17" t="inlineStr">
+        <is>
+          <t>Fell ~18% from its 10/9 record on AI-debt worries. Still tied to AI capex like the chip names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>UNP</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Union Pacific</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Railroad</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>RICH -11% (high)</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>AT RISK</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>301.93</v>
+      </c>
+      <c r="K33" s="7" t="n">
+        <v>287.39</v>
+      </c>
+      <c r="L33" s="7" t="n">
+        <v>269.98</v>
+      </c>
+      <c r="M33" s="7" t="n">
+        <v>334.65</v>
+      </c>
+      <c r="N33" s="23" t="n">
+        <v>19</v>
+      </c>
+      <c r="O33" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="P33" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>Reported 10/22</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="n"/>
+      <c r="S33" s="12">
+        <f>J33/L33-1</f>
+        <v/>
+      </c>
+      <c r="T33" s="12">
+        <f>J33/K33-1</f>
+        <v/>
+      </c>
+      <c r="U33" s="9">
+        <f>L33*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V33" s="9">
+        <f>L33*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W33" s="9">
+        <f>L33*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X33" s="12">
+        <f>J33/W33-1</f>
+        <v/>
+      </c>
+      <c r="Y33" s="12">
+        <f>IF(N(M33)&gt;0,M33/W33-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z33" s="9">
+        <f>U33</f>
+        <v/>
+      </c>
+      <c r="AA33" s="15">
+        <f>IFERROR(IF(N(M33)&gt;W33,(M33-W33)/(W33-Z33),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB33" s="24">
+        <f>IFERROR(N33/(N33+O33+P33),"")</f>
+        <v/>
+      </c>
+      <c r="AC33" s="16">
+        <f>IF(D33="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R33),Inputs!$B$5&lt;R33,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R33,"m/d"),IF(J33&lt;U33,"BELOW ZONE: wait for 200-day reclaim",IF(J33&gt;V33,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q33),AND(Q33&gt;Inputs!$B$5,Q33-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M33)&lt;=J33,"IN ZONE: analysts see no upside",IF(J33&lt;=W33,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD33" s="17" t="inlineStr">
+        <is>
+          <t>Norfolk Southern merger under STB review, close expected 2H 2027. Disruption quant flags AT RISK: check why.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Vertex Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Biotech</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>RICH -11% (high)</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>INNOVATING</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>540</v>
+      </c>
+      <c r="K34" s="7" t="n">
+        <v>522.64</v>
+      </c>
+      <c r="L34" s="7" t="n">
+        <v>478.62</v>
+      </c>
+      <c r="M34" s="7" t="n">
+        <v>575.96</v>
+      </c>
+      <c r="N34" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="O34" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="P34" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q34" s="8" t="n">
+        <v>46328</v>
+      </c>
+      <c r="R34" s="5" t="n"/>
+      <c r="S34" s="12">
+        <f>J34/L34-1</f>
+        <v/>
+      </c>
+      <c r="T34" s="12">
+        <f>J34/K34-1</f>
+        <v/>
+      </c>
+      <c r="U34" s="9">
+        <f>L34*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V34" s="9">
+        <f>L34*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W34" s="9">
+        <f>L34*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X34" s="12">
+        <f>J34/W34-1</f>
+        <v/>
+      </c>
+      <c r="Y34" s="12">
+        <f>IF(N(M34)&gt;0,M34/W34-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z34" s="9">
+        <f>U34</f>
+        <v/>
+      </c>
+      <c r="AA34" s="15">
+        <f>IFERROR(IF(N(M34)&gt;W34,(M34-W34)/(W34-Z34),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB34" s="24">
+        <f>IFERROR(N34/(N34+O34+P34),"")</f>
+        <v/>
+      </c>
+      <c r="AC34" s="16">
+        <f>IF(D34="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R34),Inputs!$B$5&lt;R34,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R34,"m/d"),IF(J34&lt;U34,"BELOW ZONE: wait for 200-day reclaim",IF(J34&gt;V34,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q34),AND(Q34&gt;Inputs!$B$5,Q34-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M34)&lt;=J34,"IN ZONE: analysts see no upside",IF(J34&lt;=W34,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD34" s="17" t="inlineStr">
+        <is>
+          <t>Cystic fibrosis franchise; $10B Crinetics deal pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>CPAY</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Corpay</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>397.97</v>
+      </c>
+      <c r="K35" s="7" t="n">
+        <v>403.45</v>
+      </c>
+      <c r="L35" s="7" t="n">
+        <v>355.07</v>
+      </c>
+      <c r="M35" s="7" t="n">
+        <v>458.81</v>
+      </c>
+      <c r="N35" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="O35" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P35" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="8" t="n">
+        <v>46330</v>
+      </c>
+      <c r="R35" s="5" t="n"/>
+      <c r="S35" s="12">
+        <f>J35/L35-1</f>
+        <v/>
+      </c>
+      <c r="T35" s="12">
+        <f>J35/K35-1</f>
+        <v/>
+      </c>
+      <c r="U35" s="9">
+        <f>L35*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V35" s="9">
+        <f>L35*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W35" s="9">
+        <f>L35*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X35" s="12">
+        <f>J35/W35-1</f>
+        <v/>
+      </c>
+      <c r="Y35" s="12">
+        <f>IF(N(M35)&gt;0,M35/W35-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z35" s="9">
+        <f>U35</f>
+        <v/>
+      </c>
+      <c r="AA35" s="15">
+        <f>IFERROR(IF(N(M35)&gt;W35,(M35-W35)/(W35-Z35),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB35" s="24">
+        <f>IFERROR(N35/(N35+O35+P35),"")</f>
+        <v/>
+      </c>
+      <c r="AC35" s="16">
+        <f>IF(D35="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R35),Inputs!$B$5&lt;R35,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R35,"m/d"),IF(J35&lt;U35,"BELOW ZONE: wait for 200-day reclaim",IF(J35&gt;V35,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q35),AND(Q35&gt;Inputs!$B$5,Q35-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M35)&lt;=J35,"IN ZONE: analysts see no upside",IF(J35&lt;=W35,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD35" s="17" t="inlineStr">
+        <is>
+          <t>Rev +21%, raised 2026 guidance in Aug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>AFRM</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Affirm</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Payments / BNPL</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="J36" s="7" t="n">
+        <v>74.84</v>
+      </c>
+      <c r="K36" s="7" t="n">
+        <v>73.08</v>
+      </c>
+      <c r="L36" s="7" t="n">
+        <v>66.51000000000001</v>
+      </c>
+      <c r="M36" s="7" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="N36" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="O36" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="P36" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="8" t="n">
+        <v>46331</v>
+      </c>
+      <c r="R36" s="8" t="n">
+        <v>46340</v>
+      </c>
+      <c r="S36" s="12">
+        <f>J36/L36-1</f>
+        <v/>
+      </c>
+      <c r="T36" s="12">
+        <f>J36/K36-1</f>
+        <v/>
+      </c>
+      <c r="U36" s="9">
+        <f>L36*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V36" s="9">
+        <f>L36*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W36" s="9">
+        <f>L36*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X36" s="12">
+        <f>J36/W36-1</f>
+        <v/>
+      </c>
+      <c r="Y36" s="12">
+        <f>IF(N(M36)&gt;0,M36/W36-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z36" s="9">
+        <f>U36</f>
+        <v/>
+      </c>
+      <c r="AA36" s="15">
+        <f>IFERROR(IF(N(M36)&gt;W36,(M36-W36)/(W36-Z36),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB36" s="24">
+        <f>IFERROR(N36/(N36+O36+P36),"")</f>
+        <v/>
+      </c>
+      <c r="AC36" s="16">
+        <f>IF(D36="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R36),Inputs!$B$5&lt;R36,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R36,"m/d"),IF(J36&lt;U36,"BELOW ZONE: wait for 200-day reclaim",IF(J36&gt;V36,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q36),AND(Q36&gt;Inputs!$B$5,Q36-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M36)&lt;=J36,"IN ZONE: analysts see no upside",IF(J36&lt;=W36,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD36" s="17" t="inlineStr">
+        <is>
+          <t>Sold at a loss 10/14: wash-sale lock to 11/14. Missed EPS the last 3 quarters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Consumer tech</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>EXPENSIVE -37% (high)</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>INNOVATING</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>348.91</v>
+      </c>
+      <c r="K37" s="7" t="n">
+        <v>332.27</v>
+      </c>
+      <c r="L37" s="7" t="n">
+        <v>296.11</v>
+      </c>
+      <c r="M37" s="7" t="n">
+        <v>334.65</v>
+      </c>
+      <c r="N37" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="O37" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="P37" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q37" s="8" t="n">
+        <v>46328</v>
+      </c>
+      <c r="R37" s="5" t="n"/>
+      <c r="S37" s="12">
+        <f>J37/L37-1</f>
+        <v/>
+      </c>
+      <c r="T37" s="12">
+        <f>J37/K37-1</f>
+        <v/>
+      </c>
+      <c r="U37" s="9">
+        <f>L37*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V37" s="9">
+        <f>L37*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W37" s="9">
+        <f>L37*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X37" s="12">
+        <f>J37/W37-1</f>
+        <v/>
+      </c>
+      <c r="Y37" s="12">
+        <f>IF(N(M37)&gt;0,M37/W37-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z37" s="9">
+        <f>U37</f>
+        <v/>
+      </c>
+      <c r="AA37" s="15">
+        <f>IFERROR(IF(N(M37)&gt;W37,(M37-W37)/(W37-Z37),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB37" s="24">
+        <f>IFERROR(N37/(N37+O37+P37),"")</f>
+        <v/>
+      </c>
+      <c r="AC37" s="16">
+        <f>IF(D37="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R37),Inputs!$B$5&lt;R37,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R37,"m/d"),IF(J37&lt;U37,"BELOW ZONE: wait for 200-day reclaim",IF(J37&gt;V37,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q37),AND(Q37&gt;Inputs!$B$5,Q37-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M37)&lt;=J37,"IN ZONE: analysts see no upside",IF(J37&lt;=W37,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD37" s="17" t="inlineStr">
+        <is>
+          <t>Analyst mean target is BELOW price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Mastercard</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>New industry</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>FAIR +4% (high)</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>STABLE</t>
+        </is>
+      </c>
+      <c r="J38" s="7" t="n">
+        <v>635.7</v>
+      </c>
+      <c r="K38" s="7" t="n">
+        <v>584.9400000000001</v>
+      </c>
+      <c r="L38" s="7" t="n">
+        <v>535.15</v>
+      </c>
+      <c r="M38" s="7" t="n">
+        <v>695.83</v>
+      </c>
+      <c r="N38" s="23" t="n">
+        <v>39</v>
+      </c>
+      <c r="O38" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P38" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" s="8" t="inlineStr">
+        <is>
+          <t>Reported 10/29</t>
+        </is>
+      </c>
+      <c r="R38" s="5" t="n"/>
+      <c r="S38" s="12">
+        <f>J38/L38-1</f>
+        <v/>
+      </c>
+      <c r="T38" s="12">
+        <f>J38/K38-1</f>
+        <v/>
+      </c>
+      <c r="U38" s="9">
+        <f>L38*(1+Inputs!$B$17)</f>
+        <v/>
+      </c>
+      <c r="V38" s="9">
+        <f>L38*(1+Inputs!$B$18)</f>
+        <v/>
+      </c>
+      <c r="W38" s="9">
+        <f>L38*(1+Inputs!$B$19)</f>
+        <v/>
+      </c>
+      <c r="X38" s="12">
+        <f>J38/W38-1</f>
+        <v/>
+      </c>
+      <c r="Y38" s="12">
+        <f>IF(N(M38)&gt;0,M38/W38-1,"")</f>
+        <v/>
+      </c>
+      <c r="Z38" s="9">
+        <f>U38</f>
+        <v/>
+      </c>
+      <c r="AA38" s="15">
+        <f>IFERROR(IF(N(M38)&gt;W38,(M38-W38)/(W38-Z38),""),"")</f>
+        <v/>
+      </c>
+      <c r="AB38" s="24">
+        <f>IFERROR(N38/(N38+O38+P38),"")</f>
+        <v/>
+      </c>
+      <c r="AC38" s="16">
+        <f>IF(D38="HELD","HELD: see Holdings sheet",IF(IF(ISNUMBER(R38),Inputs!$B$5&lt;R38,FALSE),"WASH-SALE LOCK until "&amp;TEXT(R38,"m/d"),IF(J38&lt;U38,"BELOW ZONE: wait for 200-day reclaim",IF(J38&gt;V38,"ABOVE ZONE: extended, wait",IF(IF(ISNUMBER(Q38),AND(Q38&gt;Inputs!$B$5,Q38-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"IN ZONE: earnings soon, wait",IF(N(M38)&lt;=J38,"IN ZONE: analysts see no upside",IF(J38&lt;=W38,"IN ZONE: at/below buy target - research","IN ZONE: research")))))))</f>
+        <v/>
+      </c>
+      <c r="AD38" s="17" t="inlineStr">
+        <is>
+          <t>Q3 beat (adj EPS $5.31 vs $5.15, rev +14%). Near record high: 19% above its 200-day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>COUNT</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n"/>
-      <c r="C30" s="18" t="n"/>
-      <c r="D30" s="18" t="n"/>
-      <c r="E30" s="18" t="n"/>
-      <c r="F30" s="18" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="18" t="n"/>
-      <c r="I30" s="18" t="n"/>
-      <c r="J30" s="18" t="n"/>
-      <c r="K30" s="18" t="n"/>
-      <c r="L30" s="18" t="n"/>
-      <c r="M30" s="18" t="n"/>
-      <c r="N30" s="18" t="n"/>
-      <c r="O30" s="18" t="n"/>
-      <c r="P30" s="18" t="n"/>
-      <c r="Q30" s="18" t="n"/>
-      <c r="R30" s="18" t="n"/>
-      <c r="S30" s="18" t="n"/>
-      <c r="T30" s="18" t="n"/>
-      <c r="U30" s="18" t="n"/>
-      <c r="V30" s="18" t="n"/>
-      <c r="W30" s="18" t="n"/>
-      <c r="X30" s="18" t="n"/>
-      <c r="Y30" s="18" t="n"/>
-      <c r="Z30" s="18" t="n"/>
-      <c r="AA30" s="18" t="n"/>
-      <c r="AB30" s="18" t="n"/>
-      <c r="AC30" s="18">
-        <f>COUNTIF(AC5:AC28,"IN ZONE*")&amp;" in zone, "&amp;COUNTIF(AC5:AC28,"BELOW*")&amp;" below, "&amp;COUNTIF(AC5:AC28,"ABOVE*")&amp;" above"</f>
-        <v/>
-      </c>
-      <c r="AD30" s="18" t="n"/>
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="18" t="n"/>
+      <c r="D40" s="18" t="n"/>
+      <c r="E40" s="18" t="n"/>
+      <c r="F40" s="18" t="n"/>
+      <c r="G40" s="18" t="n"/>
+      <c r="H40" s="18" t="n"/>
+      <c r="I40" s="18" t="n"/>
+      <c r="J40" s="18" t="n"/>
+      <c r="K40" s="18" t="n"/>
+      <c r="L40" s="18" t="n"/>
+      <c r="M40" s="18" t="n"/>
+      <c r="N40" s="18" t="n"/>
+      <c r="O40" s="18" t="n"/>
+      <c r="P40" s="18" t="n"/>
+      <c r="Q40" s="18" t="n"/>
+      <c r="R40" s="18" t="n"/>
+      <c r="S40" s="18" t="n"/>
+      <c r="T40" s="18" t="n"/>
+      <c r="U40" s="18" t="n"/>
+      <c r="V40" s="18" t="n"/>
+      <c r="W40" s="18" t="n"/>
+      <c r="X40" s="18" t="n"/>
+      <c r="Y40" s="18" t="n"/>
+      <c r="Z40" s="18" t="n"/>
+      <c r="AA40" s="18" t="n"/>
+      <c r="AB40" s="18" t="n"/>
+      <c r="AC40" s="18">
+        <f>COUNTIF(AC5:AC38,"IN ZONE*")&amp;" in zone, "&amp;COUNTIF(AC5:AC38,"BELOW*")&amp;" below, "&amp;COUNTIF(AC5:AC38,"ABOVE*")&amp;" above"</f>
+        <v/>
+      </c>
+      <c r="AD40" s="18" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:AD28"/>
-  <conditionalFormatting sqref="AC5:AC28">
+  <autoFilter ref="A4:AD38"/>
+  <conditionalFormatting sqref="AC5:AC38">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>LEFT(AC5,7)="IN ZONE"</formula>
     </cfRule>
@@ -7220,7 +8358,7 @@
       <formula>LEFT(AC5,5)="BELOW"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I28">
+  <conditionalFormatting sqref="I5:I38">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
       <formula>"AT RISK"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Joint tracker: build from joint_tracker_data.json; routine step 4f refreshes it (prompt v8)
build_joint_tracker.py now joins joint_tracker_data.json (positions, prices,
SMAs, 60-day range, analyst ratings, earnings) with the price-target,
valuation, setup, re-buy and wash-sale files. The Quality @ 200-day prompt v8
adds step 4f to refresh the data and rebuild the workbook each run. Watchlist
now shows wash-sale locks from wash_sale_watch.json (AVGO, SKHY to 11/22).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XBawetM5mpZm52AQxpa6eR
</commit_message>
<xml_diff>
--- a/joint_portfolio_tracker.xlsx
+++ b/joint_portfolio_tracker.xlsx
@@ -608,13 +608,18 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Close date:</t>
+          <t>Close 2026-10-29</t>
         </is>
       </c>
       <c r="D3" s="2">
         <f>Inputs!$B$5</f>
         <v/>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Not priced (check in the app): EPIX^</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -649,7 +654,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -895,7 +900,7 @@
       </c>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>RICH</t>
+          <t>RICH -14% (low)</t>
         </is>
       </c>
       <c r="T6" s="5" t="inlineStr">
@@ -905,7 +910,7 @@
       </c>
       <c r="U6" s="8" t="inlineStr">
         <is>
-          <t>Not in next 30d</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V6" s="9">
@@ -988,7 +993,11 @@
         <f>IF(W6&lt;100,"DUST: clean up",IF(V6&lt;AK6,"REVIEW: below support / max loss",IF(AND(N(Q6)&gt;0,V6&gt;=AH6),"SELL 2nd TRIM, trail the rest",IF(AND(N(Q6)&gt;0,V6&gt;=AG6),"TRIM 1/3 + thesis re-check",IF(AA6&gt;IF(ISNUMBER(SEARCH("Lev",C6)),Inputs!$B$15,Inputs!$B$14),"OVERWEIGHT: trim to cap",IF(IF(ISNUMBER(U6),AND(U6&gt;Inputs!$B$5,U6-Inputs!$B$5&lt;=Inputs!$B$16),FALSE),"HOLD: earnings soon",IF(N(Q6)=0,"HOLD: no target","HOLD")))))))</f>
         <v/>
       </c>
-      <c r="AP6" s="17" t="inlineStr"/>
+      <c r="AP6" s="17" t="inlineStr">
+        <is>
+          <t>Already held (~15% of the joint account).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1057,7 +1066,7 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>DEEP VALUE (low conf.)</t>
+          <t>DEEP VALUE +100% (low)</t>
         </is>
       </c>
       <c r="T7" s="5" t="inlineStr">
@@ -1384,12 +1393,12 @@
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U9" s="8" t="inlineStr">
+        <is>
           <t>n/a</t>
-        </is>
-      </c>
-      <c r="U9" s="8" t="inlineStr">
-        <is>
-          <t>Not in next 30d</t>
         </is>
       </c>
       <c r="V9" s="9">
@@ -1539,7 +1548,7 @@
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE (low conf.)</t>
+          <t>EXPENSIVE -50% (low)</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
@@ -1701,7 +1710,7 @@
       </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE</t>
+          <t>EXPENSIVE -27% (med)</t>
         </is>
       </c>
       <c r="T11" s="5" t="inlineStr">
@@ -1863,7 +1872,7 @@
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>RICH</t>
+          <t>RICH -13% (med)</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
@@ -1873,7 +1882,7 @@
       </c>
       <c r="U12" s="8" t="inlineStr">
         <is>
-          <t>Not in next 30d</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V12" s="9">
@@ -1965,12 +1974,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Ascendis Pharma</t>
+          <t>ServiceNow</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -1980,45 +1989,45 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Biotech</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>20</v>
+        <v>46.881838</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>226.14</v>
+        <v>103.9</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>253</v>
+        <v>109.67</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>253</v>
+        <v>109.23</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>242.38</v>
+        <v>139.99</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>237.93</v>
+        <v>115.34</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>219.52</v>
+        <v>111.8</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>272.47</v>
+        <v>159.5</v>
       </c>
       <c r="M13" s="7" t="n">
-        <v>282.15</v>
+        <v>192.97</v>
       </c>
       <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n">
-        <v>302.81</v>
+        <v>158.78</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>302</v>
+        <v>195.5</v>
       </c>
       <c r="Q13" s="7" t="n">
-        <v>302.4</v>
+        <v>177.14</v>
       </c>
       <c r="R13" s="5" t="inlineStr">
         <is>
@@ -2027,16 +2036,18 @@
       </c>
       <c r="S13" s="5" t="inlineStr">
         <is>
+          <t>DEEP VALUE +87% (low)</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>DISRUPTOR</t>
+        </is>
+      </c>
+      <c r="U13" s="8" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
-      </c>
-      <c r="T13" s="5" t="inlineStr">
-        <is>
-          <t>DISRUPTOR</t>
-        </is>
-      </c>
-      <c r="U13" s="8" t="n">
-        <v>46337</v>
       </c>
       <c r="V13" s="9">
         <f>IF(AND(Inputs!$B$6="After-hours",N(H13)&gt;0),H13,G13)</f>
@@ -2120,19 +2131,19 @@
       </c>
       <c r="AP13" s="17" t="inlineStr">
         <is>
-          <t>Earnings date unverified.</t>
+          <t>Closed below its 60-day low on 10/29.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ASND</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>ServiceNow</t>
+          <t>Ascendis Pharma</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2142,45 +2153,45 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Biotech</t>
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>46.881838</v>
+        <v>20</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>103.9</v>
+        <v>226.14</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>109.67</v>
+        <v>253</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>109.23</v>
+        <v>253</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>139.99</v>
+        <v>242.38</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>115.34</v>
+        <v>237.93</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>111.8</v>
+        <v>219.52</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>159.5</v>
+        <v>272.47</v>
       </c>
       <c r="M14" s="7" t="n">
-        <v>192.97</v>
+        <v>282.15</v>
       </c>
       <c r="N14" s="7" t="n"/>
       <c r="O14" s="7" t="n">
-        <v>158.78</v>
+        <v>302.81</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>195.5</v>
+        <v>302</v>
       </c>
       <c r="Q14" s="7" t="n">
-        <v>177.14</v>
+        <v>302.4</v>
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
@@ -2189,7 +2200,7 @@
       </c>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>DEEP VALUE (low conf.)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
@@ -2197,10 +2208,8 @@
           <t>DISRUPTOR</t>
         </is>
       </c>
-      <c r="U14" s="8" t="inlineStr">
-        <is>
-          <t>Not in next 30d</t>
-        </is>
+      <c r="U14" s="8" t="n">
+        <v>46337</v>
       </c>
       <c r="V14" s="9">
         <f>IF(AND(Inputs!$B$6="After-hours",N(H14)&gt;0),H14,G14)</f>
@@ -2284,7 +2293,7 @@
       </c>
       <c r="AP14" s="17" t="inlineStr">
         <is>
-          <t>Closed below its 60-day low on 10/29.</t>
+          <t>Earnings date unverified.</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2364,7 @@
       </c>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE</t>
+          <t>EXPENSIVE -36% (low)</t>
         </is>
       </c>
       <c r="T15" s="5" t="inlineStr">
@@ -2515,7 +2524,7 @@
       </c>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE</t>
+          <t>EXPENSIVE -35% (med)</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
@@ -2525,7 +2534,7 @@
       </c>
       <c r="U16" s="8" t="inlineStr">
         <is>
-          <t>Not in next 30d</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V16" s="9">
@@ -2679,7 +2688,7 @@
       </c>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>EXPENSIVE (low conf.)</t>
+          <t>EXPENSIVE -50% (low)</t>
         </is>
       </c>
       <c r="T17" s="5" t="inlineStr">
@@ -2846,7 +2855,7 @@
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U18" s="8" t="n">
@@ -3165,7 +3174,7 @@
       </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>RICH</t>
+          <t>RICH -13% (low)</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr">
@@ -3175,7 +3184,7 @@
       </c>
       <c r="U20" s="8" t="inlineStr">
         <is>
-          <t>Not in next 30d</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V20" s="9">
@@ -3499,7 +3508,7 @@
       </c>
       <c r="U22" s="8" t="inlineStr">
         <is>
-          <t>Not in next 30d</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V22" s="9">
@@ -3591,64 +3600,58 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>QQQI</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Robinhood Markets</t>
+          <t>NEOS Nasdaq-100 Income</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>ETF</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Brokerage</t>
+          <t>Nasdaq-100 covered call</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.010482</v>
+        <v>0.567476</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>90.63</v>
+        <v>53.83</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>91.59</v>
+        <v>53.42</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>87.37</v>
+        <v>52.61</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>108.69</v>
+        <v>54.72</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>92.76000000000001</v>
+        <v>54.18</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>89.15000000000001</v>
+        <v>52.36</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>126.74</v>
+        <v>56.84</v>
       </c>
       <c r="M23" s="7" t="n">
-        <v>150.47</v>
+        <v>57.84</v>
       </c>
       <c r="N23" s="7" t="n"/>
-      <c r="O23" s="7" t="n">
-        <v>133.63</v>
-      </c>
-      <c r="P23" s="7" t="n">
-        <v>145</v>
-      </c>
-      <c r="Q23" s="7" t="n">
-        <v>139.31</v>
-      </c>
+      <c r="O23" s="7" t="n"/>
+      <c r="P23" s="7" t="n"/>
+      <c r="Q23" s="7" t="n"/>
       <c r="R23" s="5" t="inlineStr">
         <is>
-          <t>MED</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="S23" s="5" t="inlineStr">
@@ -3658,12 +3661,12 @@
       </c>
       <c r="T23" s="5" t="inlineStr">
         <is>
-          <t>DISRUPTOR</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U23" s="8" t="inlineStr">
         <is>
-          <t>Not in next 30d</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="V23" s="9">
@@ -3748,7 +3751,7 @@
       </c>
       <c r="AP23" s="17" t="inlineStr">
         <is>
-          <t>Fractional leftover (&lt;$1).</t>
+          <t>Fractional leftover (~$30).</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3819,7 @@
       </c>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U24" s="8" t="inlineStr">
@@ -3913,68 +3916,74 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>QQQI</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>NEOS Nasdaq-100 Income</t>
+          <t>Robinhood Markets</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>ETF</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Nasdaq-100 covered call</t>
+          <t>Brokerage</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0.567476</v>
+        <v>0.010482</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>53.83</v>
+        <v>90.63</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>53.42</v>
+        <v>91.59</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>52.61</v>
+        <v>87.37</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>54.72</v>
+        <v>108.69</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>54.18</v>
+        <v>92.76000000000001</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>52.36</v>
+        <v>89.15000000000001</v>
       </c>
       <c r="L25" s="7" t="n">
-        <v>56.84</v>
+        <v>126.74</v>
       </c>
       <c r="M25" s="7" t="n">
-        <v>57.84</v>
+        <v>150.47</v>
       </c>
       <c r="N25" s="7" t="n"/>
-      <c r="O25" s="7" t="n"/>
-      <c r="P25" s="7" t="n"/>
-      <c r="Q25" s="7" t="n"/>
+      <c r="O25" s="7" t="n">
+        <v>133.63</v>
+      </c>
+      <c r="P25" s="7" t="n">
+        <v>145</v>
+      </c>
+      <c r="Q25" s="7" t="n">
+        <v>139.31</v>
+      </c>
       <c r="R25" s="5" t="inlineStr">
         <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="S25" s="5" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
       <c r="T25" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>DISRUPTOR</t>
         </is>
       </c>
       <c r="U25" s="8" t="inlineStr">
@@ -4064,7 +4073,7 @@
       </c>
       <c r="AP25" s="17" t="inlineStr">
         <is>
-          <t>Fractional leftover (~$30).</t>
+          <t>Fractional leftover (&lt;$1).</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4285,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -4443,7 +4452,7 @@
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Feb 11 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R5" s="5" t="n"/>
@@ -4534,7 +4543,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>DISRUPTOR</t>
+          <t>INNOVATING</t>
         </is>
       </c>
       <c r="J6" s="7" t="n">
@@ -4560,7 +4569,7 @@
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>Jan 26 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R6" s="5" t="n"/>
@@ -4678,7 +4687,9 @@
       <c r="Q7" s="8" t="n">
         <v>46365</v>
       </c>
-      <c r="R7" s="5" t="n"/>
+      <c r="R7" s="8" t="n">
+        <v>46348</v>
+      </c>
       <c r="S7" s="12">
         <f>J7/L7-1</f>
         <v/>
@@ -4996,7 +5007,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>INNOVATING</t>
+          <t>STABLE</t>
         </is>
       </c>
       <c r="J10" s="7" t="n">
@@ -5022,7 +5033,7 @@
       </c>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Jan 26 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R10" s="5" t="n"/>
@@ -5113,7 +5124,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>DISRUPTOR</t>
+          <t>INNOVATING</t>
         </is>
       </c>
       <c r="J11" s="7" t="n">
@@ -5342,7 +5353,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -5373,10 +5384,12 @@
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>Feb 9 (unverified)</t>
-        </is>
-      </c>
-      <c r="R13" s="5" t="n"/>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="R13" s="8" t="n">
+        <v>46354</v>
+      </c>
       <c r="S13" s="12">
         <f>J13/L13-1</f>
         <v/>
@@ -5423,7 +5436,7 @@
       </c>
       <c r="AD13" s="17" t="inlineStr">
         <is>
-          <t>Held as a fractional leftover.</t>
+          <t>Fractional leftover (&lt;$1).</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5618,7 @@
       </c>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>Dec 10 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R15" s="5" t="n"/>
@@ -5700,7 +5713,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>DISRUPTOR</t>
+          <t>INNOVATING</t>
         </is>
       </c>
       <c r="J16" s="7" t="n">
@@ -5726,10 +5739,12 @@
       </c>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>Jan 27 (unverified)</t>
-        </is>
-      </c>
-      <c r="R16" s="5" t="n"/>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="n">
+        <v>46354</v>
+      </c>
       <c r="S16" s="12">
         <f>J16/L16-1</f>
         <v/>
@@ -5843,7 +5858,7 @@
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Feb 19 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R17" s="5" t="n"/>
@@ -6071,7 +6086,7 @@
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>Nov 5 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R19" s="5" t="n"/>
@@ -6184,7 +6199,7 @@
       </c>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Jan 28 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R20" s="5" t="n"/>
@@ -6301,7 +6316,7 @@
       </c>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>Feb 22 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R21" s="5" t="n"/>
@@ -6396,7 +6411,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>DISRUPTOR</t>
+          <t>INNOVATING</t>
         </is>
       </c>
       <c r="J22" s="7" t="n">
@@ -6422,7 +6437,7 @@
       </c>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>Feb 17 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R22" s="5" t="n"/>
@@ -6472,7 +6487,7 @@
       </c>
       <c r="AD22" s="17" t="inlineStr">
         <is>
-          <t>Already held (20 sh).</t>
+          <t>Target agreement LOW: fundamental and Robinhood targets 35% apart.</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6554,7 @@
       </c>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>Jan 22 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R23" s="5" t="n"/>
@@ -6630,7 +6645,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>AT RISK</t>
+          <t>STABLE</t>
         </is>
       </c>
       <c r="J24" s="7" t="n">
@@ -6656,7 +6671,7 @@
       </c>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>Reported 10/29</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R24" s="5" t="n"/>
@@ -6773,10 +6788,12 @@
       </c>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>Feb 13 (unverified)</t>
-        </is>
-      </c>
-      <c r="R25" s="5" t="n"/>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="R25" s="8" t="n">
+        <v>46348</v>
+      </c>
       <c r="S25" s="12">
         <f>J25/L25-1</f>
         <v/>
@@ -6890,7 +6907,7 @@
       </c>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>Feb 11 (unverified)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R26" s="5" t="n"/>
@@ -6977,7 +6994,7 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>AT RISK</t>
         </is>
       </c>
       <c r="J27" s="7" t="n">
@@ -7081,12 +7098,12 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>EXPENSIVE -50% (low)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>INNOVATING</t>
         </is>
       </c>
       <c r="J28" s="7" t="n">
@@ -7112,7 +7129,7 @@
       </c>
       <c r="Q28" s="8" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R28" s="8" t="n">
@@ -7193,7 +7210,7 @@
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Malls REIT</t>
+          <t>0 EXTENDED</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
@@ -7277,7 +7294,7 @@
       </c>
       <c r="AD29" s="17" t="inlineStr">
         <is>
-          <t>Only new name already inside the buy zone. Analysts mostly Hold.</t>
+          <t>Malls REIT. Only new name already inside the buy zone. Analysts mostly Hold.</t>
         </is>
       </c>
     </row>
@@ -7311,7 +7328,7 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>RICH -11% (med)</t>
+          <t>RICH -10% (med)</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
@@ -7390,7 +7407,7 @@
       </c>
       <c r="AD30" s="17" t="inlineStr">
         <is>
-          <t>Rev +20%, net margin 23%. 2-for-1 split Aug 2026.</t>
+          <t>Consumer staples. Rev +20%, net margin 23%. 2-for-1 split Aug 2026.</t>
         </is>
       </c>
     </row>
@@ -7424,7 +7441,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>DEEP VALUE (low conf.)</t>
+          <t>DEEP VALUE +100% (low)</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -7455,7 +7472,7 @@
       </c>
       <c r="Q31" s="8" t="inlineStr">
         <is>
-          <t>Reported 10/29</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R31" s="5" t="n"/>
@@ -7505,7 +7522,7 @@
       </c>
       <c r="AD31" s="17" t="inlineStr">
         <is>
-          <t>Q3 GAAP loss -$3.86/sh from a one-time $1.23B Vega IPR&amp;D charge; revenue +14%. Analysts split Buy/Hold.</t>
+          <t>Biotech. Q3 GAAP loss -$3.86/sh from a one-time $1.23B Vega IPR&amp;D charge; revenue +14%. Analysts split Buy/Hold.</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7635,7 @@
       </c>
       <c r="AD32" s="17" t="inlineStr">
         <is>
-          <t>Fell ~18% from its 10/9 record on AI-debt worries. Still tied to AI capex like the chip names.</t>
+          <t>AI networking. Fell ~18% from its 10/9 record on AI-debt worries. Still tied to AI capex like the chip names.</t>
         </is>
       </c>
     </row>
@@ -7683,7 +7700,7 @@
       </c>
       <c r="Q33" s="8" t="inlineStr">
         <is>
-          <t>Reported 10/22</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R33" s="5" t="n"/>
@@ -7733,7 +7750,7 @@
       </c>
       <c r="AD33" s="17" t="inlineStr">
         <is>
-          <t>Norfolk Southern merger under STB review, close expected 2H 2027. Disruption quant flags AT RISK: check why.</t>
+          <t>Railroad. Norfolk Southern merger under STB review, close expected 2H 2027. Disruption quant flags AT RISK: check why.</t>
         </is>
       </c>
     </row>
@@ -7846,7 +7863,7 @@
       </c>
       <c r="AD34" s="17" t="inlineStr">
         <is>
-          <t>Cystic fibrosis franchise; $10B Crinetics deal pending.</t>
+          <t>Biotech. Cystic fibrosis franchise; $10B Crinetics deal pending.</t>
         </is>
       </c>
     </row>
@@ -7959,7 +7976,7 @@
       </c>
       <c r="AD35" s="17" t="inlineStr">
         <is>
-          <t>Rev +21%, raised 2026 guidance in Aug.</t>
+          <t>Payments. Rev +21%, raised 2026 guidance in Aug.</t>
         </is>
       </c>
     </row>
@@ -7988,12 +8005,12 @@
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Payments / BNPL</t>
+          <t>29 MIXED</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
@@ -8074,7 +8091,7 @@
       </c>
       <c r="AD36" s="17" t="inlineStr">
         <is>
-          <t>Sold at a loss 10/14: wash-sale lock to 11/14. Missed EPS the last 3 quarters.</t>
+          <t>Payments / BNPL. Sold at a loss 10/14: wash-sale lock to 11/14. Missed EPS the last 3 quarters.</t>
         </is>
       </c>
     </row>
@@ -8187,7 +8204,7 @@
       </c>
       <c r="AD37" s="17" t="inlineStr">
         <is>
-          <t>Analyst mean target is BELOW price.</t>
+          <t>Consumer tech. Analyst mean target is BELOW price.</t>
         </is>
       </c>
     </row>
@@ -8216,7 +8233,7 @@
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>0 EXTENDED</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
@@ -8252,7 +8269,7 @@
       </c>
       <c r="Q38" s="8" t="inlineStr">
         <is>
-          <t>Reported 10/29</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="R38" s="5" t="n"/>
@@ -8302,7 +8319,7 @@
       </c>
       <c r="AD38" s="17" t="inlineStr">
         <is>
-          <t>Q3 beat (adj EPS $5.31 vs $5.15, rev +14%). Near record high: 19% above its 200-day.</t>
+          <t>Payments. Q3 beat (adj EPS $5.31 vs $5.15, rev +14%). Near record high: 19% above its 200-day.</t>
         </is>
       </c>
     </row>
@@ -8415,7 +8432,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>As-of date (close used)</t>
+          <t>As-of date (prices)</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
@@ -8423,7 +8440,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Date of the official close in the Close column.</t>
+          <t>Date of the prices in the Price column (see the Holdings header).</t>
         </is>
       </c>
     </row>
@@ -8435,12 +8452,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Price</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Close or After-hours. After-hours falls back to Close when blank.</t>
+          <t>Price or After-hours. After-hours falls back to Price when blank.</t>
         </is>
       </c>
     </row>
@@ -8642,7 +8659,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Close,After-hours"</formula1>
+      <formula1>"Price,After-hours"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8793,14 +8810,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Positions, quotes, 50/200-day SMA, 60-day range, 52-wk high, earnings dates: Robinhood (pulled 2026-10-30).</t>
+          <t>Positions, quotes, 50/200-day SMA, 60-day range, 52-wk high, analyst ratings, earnings dates: Robinhood, via joint_tracker_data.json.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Targets: joint_price_targets.json (2026-10-29). Valuation and disruption grades: valuation.json (2026-10-28/29).</t>
+          <t>Targets: joint_price_targets.json. Valuation and disruption: valuation.json. Chart setups: setups.json. Re-buy: rebuy_watch.json. Wash-sale dates: wash_sale_watch.json.</t>
         </is>
       </c>
     </row>
@@ -8817,7 +8834,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EPIX^ (25 sh, $0 cost) has no quote: likely a delisted or escrowed position. Check it in the app.</t>
+          <t>Holdings with no quote (e.g. EPIX^, 25 sh at $0 cost) are listed at the top of Holdings as Not priced.</t>
         </is>
       </c>
     </row>
@@ -8841,7 +8858,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Edit the blue cells, or update SNAPSHOT in build_joint_tracker.py and re-run it.</t>
+          <t>The Quality @ 200-day routine (step 4f) refreshes joint_tracker_data.json and rebuilds this file each weekday. Edit blue cells for what-ifs; a rebuild overwrites them.</t>
         </is>
       </c>
     </row>

</xml_diff>